<commit_message>
Update retail sector (VDS_s) 0.xlsx
</commit_message>
<xml_diff>
--- a/clustering/sepsectors/retail sector (VDS_s) 0.xlsx
+++ b/clustering/sepsectors/retail sector (VDS_s) 0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="17">
   <si>
     <t>sector</t>
   </si>
@@ -68,6 +68,9 @@
   <si>
     <t>нижний кластер:</t>
   </si>
+  <si>
+    <t>разница</t>
+  </si>
 </sst>
 </file>
 
@@ -76,7 +79,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -96,6 +99,15 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -135,7 +147,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -152,6 +164,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -455,7 +468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="93" customWidth="1"/>
@@ -773,7 +786,7 @@
         <v>4872251.3082260424</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>14</v>
       </c>
@@ -794,7 +807,7 @@
         <v>1.0257590125276369E-3</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>15</v>
       </c>
@@ -815,11 +828,833 @@
         <v>4.3731190154563726E-4</v>
       </c>
     </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D22" s="4">
+        <v>1252686.154182706</v>
+      </c>
+      <c r="E22" s="4">
+        <v>9796.3168782600005</v>
+      </c>
+      <c r="F22" s="3">
+        <v>0.13430184443805829</v>
+      </c>
+      <c r="G22" s="3">
+        <v>5.218380319387952E-4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D23" s="4">
+        <v>1194490.274669243</v>
+      </c>
+      <c r="E23" s="4">
+        <v>19231.118310289999</v>
+      </c>
+      <c r="F23" s="3">
+        <v>5.2147019888250969E-3</v>
+      </c>
+      <c r="G23" s="3">
+        <v>4.9058279907476332E-4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D24" s="4">
+        <v>1165717.934645507</v>
+      </c>
+      <c r="E24" s="4">
+        <v>8785.8682089999984</v>
+      </c>
+      <c r="F24" s="3">
+        <v>1.025148686019859E-2</v>
+      </c>
+      <c r="G24" s="3">
+        <v>1.7444704536200269E-4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D25" s="4">
+        <v>1063712.5319653209</v>
+      </c>
+      <c r="E25" s="4">
+        <v>8180.2586681400007</v>
+      </c>
+      <c r="F25" s="3">
+        <v>1.6866644248961379E-2</v>
+      </c>
+      <c r="G25" s="3">
+        <v>6.3103132179727491E-4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B27" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="4">
+        <f>AVERAGE(D22:D23)</f>
+        <v>1223588.2144259745</v>
+      </c>
+      <c r="E27" s="4">
+        <f t="shared" ref="E27:G27" si="2">AVERAGE(E22:E23)</f>
+        <v>14513.717594275</v>
+      </c>
+      <c r="F27" s="3">
+        <f t="shared" si="2"/>
+        <v>6.9758273213441691E-2</v>
+      </c>
+      <c r="G27" s="3">
+        <f t="shared" si="2"/>
+        <v>5.0621041550677926E-4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B28" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" s="4">
+        <f>AVERAGE(D24:D25)</f>
+        <v>1114715.233305414</v>
+      </c>
+      <c r="E28" s="4">
+        <f t="shared" ref="E28:G28" si="3">AVERAGE(E24:E25)</f>
+        <v>8483.0634385699996</v>
+      </c>
+      <c r="F28" s="3">
+        <f t="shared" si="3"/>
+        <v>1.3559065554579985E-2</v>
+      </c>
+      <c r="G28" s="3">
+        <f t="shared" si="3"/>
+        <v>4.0273918357963879E-4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C30" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D30" s="4">
+        <f>D27/D28</f>
+        <v>1.0976688735092679</v>
+      </c>
+      <c r="E30" s="4">
+        <f t="shared" ref="E30:G30" si="4">E27/E28</f>
+        <v>1.7109052289159346</v>
+      </c>
+      <c r="F30" s="4">
+        <f t="shared" si="4"/>
+        <v>5.1447699646144658</v>
+      </c>
+      <c r="G30" s="4">
+        <f t="shared" si="4"/>
+        <v>1.2569187110314528</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D33" s="4">
+        <v>9937990.5894197039</v>
+      </c>
+      <c r="E33" s="4">
+        <v>137654.50809200999</v>
+      </c>
+      <c r="F33" s="3">
+        <v>2.451646095414645E-3</v>
+      </c>
+      <c r="G33" s="3">
+        <v>7.6188786690442915E-4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C34" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D34" s="4">
+        <v>9153211.3096406423</v>
+      </c>
+      <c r="E34" s="4">
+        <v>158802.14720132999</v>
+      </c>
+      <c r="F34" s="3">
+        <v>2.8137256066412789E-3</v>
+      </c>
+      <c r="G34" s="3">
+        <v>2.4032687441319662E-3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C35" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D35" s="4">
+        <v>8323850.3002414759</v>
+      </c>
+      <c r="E35" s="4">
+        <v>69747.682037220002</v>
+      </c>
+      <c r="F35" s="3">
+        <v>3.3950559124479012E-3</v>
+      </c>
+      <c r="G35" s="3">
+        <v>9.6936097165093425E-4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C36" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D36" s="4">
+        <v>7695797.0900557945</v>
+      </c>
+      <c r="E36" s="4">
+        <v>86242.724574749998</v>
+      </c>
+      <c r="F36" s="3">
+        <v>2.8921735657111581E-3</v>
+      </c>
+      <c r="G36" s="3">
+        <v>1.1051378185227779E-3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B38" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D38" s="4">
+        <f>AVERAGE(D33:D34)</f>
+        <v>9545600.9495301731</v>
+      </c>
+      <c r="E38" s="4">
+        <f t="shared" ref="E38:G38" si="5">AVERAGE(E33:E34)</f>
+        <v>148228.32764666999</v>
+      </c>
+      <c r="F38" s="3">
+        <f t="shared" si="5"/>
+        <v>2.6326858510279617E-3</v>
+      </c>
+      <c r="G38" s="3">
+        <f t="shared" si="5"/>
+        <v>1.5825783055181976E-3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B39" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D39" s="4">
+        <f>AVERAGE(D35:D36)</f>
+        <v>8009823.6951486357</v>
+      </c>
+      <c r="E39" s="4">
+        <f t="shared" ref="E39:G39" si="6">AVERAGE(E35:E36)</f>
+        <v>77995.203305984993</v>
+      </c>
+      <c r="F39" s="3">
+        <f t="shared" si="6"/>
+        <v>3.1436147390795297E-3</v>
+      </c>
+      <c r="G39" s="3">
+        <f t="shared" si="6"/>
+        <v>1.0372493950868561E-3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C41" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D41" s="4">
+        <f>D38/D39</f>
+        <v>1.1917367114224651</v>
+      </c>
+      <c r="E41" s="4">
+        <f t="shared" ref="E41:G41" si="7">E38/E39</f>
+        <v>1.9004800470248358</v>
+      </c>
+      <c r="F41" s="4">
+        <f t="shared" si="7"/>
+        <v>0.8374708956221617</v>
+      </c>
+      <c r="G41" s="4">
+        <f t="shared" si="7"/>
+        <v>1.5257452190518532</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C44" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D44" s="4">
+        <v>5034263.5495518269</v>
+      </c>
+      <c r="E44" s="4">
+        <v>65873.429441999993</v>
+      </c>
+      <c r="F44" s="3">
+        <v>2.9423350149191101E-3</v>
+      </c>
+      <c r="G44" s="3">
+        <v>3.4897071466789652E-4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C45" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D45" s="4">
+        <v>4961117.4365704898</v>
+      </c>
+      <c r="E45" s="4">
+        <v>63209.692581750001</v>
+      </c>
+      <c r="F45" s="3">
+        <v>4.351387458407175E-3</v>
+      </c>
+      <c r="G45" s="3">
+        <v>5.6592795928781631E-4</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C46" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D46" s="4">
+        <v>4783385.1798815951</v>
+      </c>
+      <c r="E46" s="4">
+        <v>64669.840333150009</v>
+      </c>
+      <c r="F46" s="3">
+        <v>2.0954023999737231E-3</v>
+      </c>
+      <c r="G46" s="3">
+        <v>5.9056880507593645E-4</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C47" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D47" s="4">
+        <v>4448196.0441567702</v>
+      </c>
+      <c r="E47" s="4">
+        <v>96473.926682400008</v>
+      </c>
+      <c r="F47" s="3">
+        <v>4.425446074207404E-4</v>
+      </c>
+      <c r="G47" s="3">
+        <v>2.154034060250509E-4</v>
+      </c>
+    </row>
+    <row r="49" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B49" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D49" s="4">
+        <f>AVERAGE(D44:D45)</f>
+        <v>4997690.4930611588</v>
+      </c>
+      <c r="E49" s="4">
+        <f t="shared" ref="E49:G49" si="8">AVERAGE(E44:E45)</f>
+        <v>64541.561011874997</v>
+      </c>
+      <c r="F49" s="3">
+        <f t="shared" si="8"/>
+        <v>3.6468612366631426E-3</v>
+      </c>
+      <c r="G49" s="3">
+        <f t="shared" si="8"/>
+        <v>4.5744933697785639E-4</v>
+      </c>
+    </row>
+    <row r="50" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B50" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D50" s="4">
+        <f>AVERAGE(D46:D47)</f>
+        <v>4615790.6120191831</v>
+      </c>
+      <c r="E50" s="4">
+        <f t="shared" ref="E50:G50" si="9">AVERAGE(E46:E47)</f>
+        <v>80571.883507775012</v>
+      </c>
+      <c r="F50" s="3">
+        <f t="shared" si="9"/>
+        <v>1.2689735036972318E-3</v>
+      </c>
+      <c r="G50" s="3">
+        <f t="shared" si="9"/>
+        <v>4.0298610555049367E-4</v>
+      </c>
+    </row>
+    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C52" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D52" s="4">
+        <f>D49/D50</f>
+        <v>1.0827376961267559</v>
+      </c>
+      <c r="E52" s="4">
+        <f t="shared" ref="E52:G52" si="10">E49/E50</f>
+        <v>0.80104322006630113</v>
+      </c>
+      <c r="F52" s="4">
+        <f t="shared" si="10"/>
+        <v>2.8738671264906555</v>
+      </c>
+      <c r="G52" s="4">
+        <f t="shared" si="10"/>
+        <v>1.1351491544676557</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState ref="A2:G13">
-    <sortCondition descending="1" ref="D2:D13"/>
+  <sortState ref="A22:G25">
+    <sortCondition descending="1" ref="D22:D25"/>
   </sortState>
   <conditionalFormatting sqref="D2:D13">
+    <cfRule type="colorScale" priority="32">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E13">
+    <cfRule type="colorScale" priority="31">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F13">
+    <cfRule type="colorScale" priority="30">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G13">
+    <cfRule type="colorScale" priority="29">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D17:D18">
+    <cfRule type="colorScale" priority="28">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17:E18">
+    <cfRule type="colorScale" priority="27">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F17:F18">
+    <cfRule type="colorScale" priority="26">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G17:G18">
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D22:D25">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E22:E25">
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F22:F25">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G22:G25">
+    <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D27:D28">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E27:E28">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F27:F28">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G27:G28">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D33:D36">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E33:E36">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F33:F36">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G33:G36">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D38:D39">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E38:E39">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F38:F39">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G38:G39">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D44:D47">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -831,7 +1666,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E13">
+  <conditionalFormatting sqref="E44:E47">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -843,7 +1678,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F13">
+  <conditionalFormatting sqref="F44:F47">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -855,7 +1690,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G13">
+  <conditionalFormatting sqref="G44:G47">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -867,7 +1702,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D17:D18">
+  <conditionalFormatting sqref="D49:D50">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -879,7 +1714,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E17:E18">
+  <conditionalFormatting sqref="E49:E50">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -891,7 +1726,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F17:F18">
+  <conditionalFormatting sqref="F49:F50">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -903,7 +1738,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G17:G18">
+  <conditionalFormatting sqref="G49:G50">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>